<commit_message>
add unit tests for isotope correction + fix [Na]+ corr bug
</commit_message>
<xml_diff>
--- a/tests/database/test_database.xlsx
+++ b/tests/database/test_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/msi-quant/tests/database/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/LipidQMap/tests/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2346C327-0B09-6B45-9F4F-10237ED9B5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D28BC8-6D86-1240-AAA1-5AF205BE8B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4660" yWindow="860" windowWidth="30240" windowHeight="17560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="860" windowWidth="30240" windowHeight="17560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -141,6 +141,12 @@
   </si>
   <si>
     <t>Neutral Formula</t>
+  </si>
+  <si>
+    <t>PC 32:0</t>
+  </si>
+  <si>
+    <t>C40H80NPO8</t>
   </si>
 </sst>
 </file>
@@ -196,15 +202,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -510,316 +513,302 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
-    <col min="5" max="5" width="20.5" customWidth="1"/>
-    <col min="6" max="6" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+    <col min="4" max="4" width="20.5" customWidth="1"/>
+    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
-        <v>0</v>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>21</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="4">
+      <c r="G2" s="3">
         <v>1.5</v>
       </c>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>1</v>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>36</v>
       </c>
       <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" s="1"/>
+      <c r="G3" s="3"/>
+      <c r="H3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="4"/>
-      <c r="I3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="G4" s="3"/>
+      <c r="H4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B5" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>2</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="4"/>
-      <c r="I4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="1">
+      <c r="G5" s="3"/>
+      <c r="H5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="3"/>
+      <c r="H6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="G11" s="3"/>
+      <c r="H11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="3"/>
+      <c r="H12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>2</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="4"/>
-      <c r="I5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="4"/>
-      <c r="I6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7" s="1">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="4"/>
-      <c r="I7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" t="s">
-        <v>2</v>
-      </c>
-      <c r="E8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" s="4"/>
-      <c r="I8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="4"/>
-      <c r="I9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" t="s">
-        <v>3</v>
-      </c>
-      <c r="H10" s="4"/>
-      <c r="I10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" t="s">
-        <v>2</v>
-      </c>
-      <c r="E11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" t="s">
-        <v>4</v>
-      </c>
-      <c r="H11" s="4"/>
-      <c r="I11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
+      <c r="G13" s="3"/>
+      <c r="H13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>10</v>
       </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" t="s">
-        <v>5</v>
-      </c>
-      <c r="H12" s="4"/>
-      <c r="I12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13" s="1">
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
         <v>11</v>
       </c>
-      <c r="B13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="D14" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="4"/>
+      <c r="G14" s="3"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="K1:Q12">
-    <sortCondition ref="M1:M12"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J1:P13">
+    <sortCondition ref="L1:L13"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
add unittests, remove forbidden characters from save dir
</commit_message>
<xml_diff>
--- a/tests/database/test_database.xlsx
+++ b/tests/database/test_database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/LipidQMap/tests/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D28BC8-6D86-1240-AAA1-5AF205BE8B6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B068C2E-266D-704D-AAFE-1000C288ACC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="860" windowWidth="30240" windowHeight="17560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="42">
   <si>
     <t>ID</t>
   </si>
@@ -147,6 +147,18 @@
   </si>
   <si>
     <t>C40H80NPO8</t>
+  </si>
+  <si>
+    <t>SM 34:1</t>
+  </si>
+  <si>
+    <t>SM</t>
+  </si>
+  <si>
+    <t>[M+H]+</t>
+  </si>
+  <si>
+    <t>C39H79N2O6P</t>
   </si>
 </sst>
 </file>
@@ -513,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -793,18 +805,33 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" s="3"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>10</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C15" t="s">
         <v>11</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="3"/>
+      <c r="G15" s="3"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J1:P13">

</xml_diff>

<commit_message>
also use M-4 isotope in db correction
</commit_message>
<xml_diff>
--- a/tests/database/test_database.xlsx
+++ b/tests/database/test_database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/LipidQMap/tests/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B068C2E-266D-704D-AAFE-1000C288ACC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C1D0FE0-9C79-254B-A4D3-9599F0FE7B74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35460" yWindow="1560" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="43">
   <si>
     <t>ID</t>
   </si>
@@ -159,12 +159,18 @@
   </si>
   <si>
     <t>C39H79N2O6P</t>
+  </si>
+  <si>
+    <t>M-4 Isotope</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -214,7 +220,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -223,6 +229,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -525,19 +532,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.5" customWidth="1"/>
     <col min="4" max="4" width="20.5" customWidth="1"/>
     <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5" customWidth="1"/>
+    <col min="7" max="7" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -554,16 +562,19 @@
         <v>19</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -578,12 +589,13 @@
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="3">
+      <c r="G2" s="1"/>
+      <c r="H2" s="3">
         <v>1.5</v>
       </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -599,13 +611,16 @@
       <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="3"/>
-      <c r="H3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="1"/>
+      <c r="H3" s="3"/>
+      <c r="I3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -621,12 +636,12 @@
       <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="3"/>
-      <c r="H4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H4" s="3"/>
+      <c r="I4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -642,12 +657,12 @@
       <c r="E5" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="3"/>
-      <c r="H5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H5" s="3"/>
+      <c r="I5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -663,12 +678,12 @@
       <c r="E6" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="3"/>
-      <c r="H6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H6" s="3"/>
+      <c r="I6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -681,12 +696,12 @@
       <c r="D7" t="s">
         <v>21</v>
       </c>
-      <c r="G7" s="3"/>
-      <c r="H7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="3"/>
+      <c r="I7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -699,12 +714,12 @@
       <c r="D8" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="3"/>
-      <c r="H8" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="3"/>
+      <c r="I8" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -717,12 +732,12 @@
       <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="3"/>
+      <c r="I9" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -735,12 +750,12 @@
       <c r="D10" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="3"/>
-      <c r="H10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H10" s="3"/>
+      <c r="I10" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -753,15 +768,15 @@
       <c r="D11" t="s">
         <v>21</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="3"/>
-      <c r="H11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H11" s="3"/>
+      <c r="I11" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>15</v>
       </c>
@@ -774,15 +789,15 @@
       <c r="D12" t="s">
         <v>21</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="3"/>
-      <c r="H12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H12" s="3"/>
+      <c r="I12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -795,15 +810,15 @@
       <c r="D13" t="s">
         <v>21</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="3"/>
-      <c r="H13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H13" s="3"/>
+      <c r="I13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>38</v>
       </c>
@@ -816,9 +831,9 @@
       <c r="D14" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="3"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>10</v>
       </c>
@@ -831,11 +846,17 @@
       <c r="D15" t="s">
         <v>12</v>
       </c>
-      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.2">
+      <c r="H17" s="4"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J1:P13">
-    <sortCondition ref="L1:L13"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="K1:Q13">
+    <sortCondition ref="M1:M13"/>
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
database column name change
</commit_message>
<xml_diff>
--- a/tests/database/test_database.xlsx
+++ b/tests/database/test_database.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/LipidQMap/tests/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{960F22E6-2DEB-EB4A-A2BE-307DCDA98479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BBD9EEE-85B0-DD40-BA44-E69BCFB55213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-35460" yWindow="1560" windowWidth="30240" windowHeight="17460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,9 +89,6 @@
     <t>IS</t>
   </si>
   <si>
-    <t>IS amount (pmol / mm2)</t>
-  </si>
-  <si>
     <t>M-2 Isotope</t>
   </si>
   <si>
@@ -164,7 +161,10 @@
     <t>M-4 Isotope</t>
   </si>
   <si>
-    <t>IS standard</t>
+    <t>Is standard</t>
+  </si>
+  <si>
+    <t>Standard amount (pmol / mm2)</t>
   </si>
 </sst>
 </file>
@@ -554,28 +554,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>17</v>
@@ -586,13 +586,13 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -607,16 +607,16 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
         <v>36</v>
       </c>
-      <c r="B3" t="s">
-        <v>37</v>
-      </c>
       <c r="C3" t="s">
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E3" t="s">
         <v>3</v>
@@ -638,13 +638,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
         <v>6</v>
@@ -662,13 +662,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
         <v>2</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
         <v>7</v>
@@ -686,13 +686,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
@@ -710,13 +710,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
         <v>2</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H7" s="1" t="b">
         <v>0</v>
@@ -731,13 +731,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H8" s="1" t="b">
         <v>0</v>
@@ -752,13 +752,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C9" t="s">
         <v>2</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H9" s="1" t="b">
         <v>0</v>
@@ -773,13 +773,13 @@
         <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" t="s">
         <v>2</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H10" s="1" t="b">
         <v>0</v>
@@ -794,13 +794,13 @@
         <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
         <v>2</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G11" t="s">
         <v>3</v>
@@ -818,13 +818,13 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G12" t="s">
         <v>4</v>
@@ -842,13 +842,13 @@
         <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C13" t="s">
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G13" t="s">
         <v>5</v>
@@ -863,16 +863,16 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s">
         <v>38</v>
       </c>
-      <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>39</v>
-      </c>
-      <c r="D14" t="s">
-        <v>40</v>
       </c>
       <c r="H14" s="1" t="b">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C15" t="s">
         <v>11</v>

</xml_diff>